<commit_message>
0.1.1: screenshots, a card-grid example app and realistic samples
The example's home screen is a grid of document cards with large
thumbnails and format badges. The sample PDF, Word report and text notes
read like real documents (the Word sample was the test fixture), the
deck carries the package's name, and the sheet stores its totals as
values. test_driver/screenshots_test.dart takes the README and pub.dev
screenshots on a phone emulator.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TntCBjAikJ5L34LJmcwdCX
</commit_message>
<xml_diff>
--- a/example/assets/samples/sales.xlsx
+++ b/example/assets/samples/sales.xlsx
@@ -490,8 +490,11 @@
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -632,13 +635,11 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B8" s="4">
-        <f>SUM(B2:B6)</f>
-        <v/>
-      </c>
-      <c r="C8" s="4">
-        <f>SUM(C2:C6)</f>
-        <v/>
+      <c r="B8" s="4" t="n">
+        <v>485</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>505</v>
       </c>
       <c r="D8" s="4" t="n"/>
       <c r="E8" s="4" t="n"/>

</xml_diff>